<commit_message>
feat(isobutanol): relocate the opt_IRR workbook to split_12d PI (log-tail) GP trial 1602
Baseline (and +/-20 % distribution) columns now hold trial 1602 of kin_opt_ethanol_isobutanol_metabolic_split_12d_pi_log-tail_gp_rb0.001-4_ib0.75-1.5_aA_burden (anchor scenario A), as written by build_opt_IRR_split12d_workbook.py, with a per-row provenance note (164 cells). This is the workbook the 2026-09-20 scenarios.SCENARIOS['opt_IRR'] pin and smoke test 9 (ethanol 0.35881 / isobutanol 1.1635, IRR 0.27299) already assume; HEAD still carried the previous trial-774 point.

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/biorefineries/isobutanol/analyses/full/parameter_distributions/parameter-distributions_corn_IBO_EtOH_opt_IRR.xlsx
+++ b/biorefineries/isobutanol/analyses/full/parameter_distributions/parameter-distributions_corn_IBO_EtOH_opt_IRR.xlsx
@@ -1404,7 +1404,7 @@
         </is>
       </c>
       <c r="E21" s="3" t="n">
-        <v>1.000993446018799</v>
+        <v>1.527675739434997</v>
       </c>
       <c r="F21" s="3" t="inlineStr">
         <is>
@@ -1412,15 +1412,19 @@
         </is>
       </c>
       <c r="G21" s="3" t="n">
-        <v>0.8007947568150389</v>
+        <v>1.222140591547997</v>
       </c>
       <c r="H21" s="3" t="n">
-        <v>1.000993446018799</v>
+        <v>1.527675739434997</v>
       </c>
       <c r="I21" s="3" t="n">
-        <v>1.201192135222558</v>
-      </c>
-      <c r="J21" s="3" t="n"/>
+        <v>1.833210887321996</v>
+      </c>
+      <c r="J21" s="3" t="inlineStr">
+        <is>
+          <t>opt_IRR: trial 1602 of kin_opt_ethanol_isobutanol_metabolic_split_12d_pi_log-tail_gp_rb0.001-4_ib0.75-1.5_aA_burden (anchor scenario A; build_opt_IRR_split12d_workbook.py)</t>
+        </is>
+      </c>
       <c r="K21" s="3" t="inlineStr">
         <is>
           <t>V406.nsk_kinetic_model._te.k_1l = x</t>
@@ -1465,7 +1469,11 @@
       <c r="I22" s="3" t="n">
         <v>1.128</v>
       </c>
-      <c r="J22" s="3" t="n"/>
+      <c r="J22" s="3" t="inlineStr">
+        <is>
+          <t>opt_IRR: trial 1602 of kin_opt_ethanol_isobutanol_metabolic_split_12d_pi_log-tail_gp_rb0.001-4_ib0.75-1.5_aA_burden (anchor scenario A; build_opt_IRR_split12d_workbook.py)</t>
+        </is>
+      </c>
       <c r="K22" s="3" t="inlineStr">
         <is>
           <t>V406.nsk_kinetic_model._te.K_1l = x</t>
@@ -1494,7 +1502,7 @@
         </is>
       </c>
       <c r="E23" s="3" t="n">
-        <v>0.9301227008430398</v>
+        <v>0.6238899523286979</v>
       </c>
       <c r="F23" s="3" t="inlineStr">
         <is>
@@ -1502,15 +1510,19 @@
         </is>
       </c>
       <c r="G23" s="3" t="n">
-        <v>0.7440981606744319</v>
+        <v>0.4991119618629584</v>
       </c>
       <c r="H23" s="3" t="n">
-        <v>0.9301227008430398</v>
+        <v>0.6238899523286979</v>
       </c>
       <c r="I23" s="3" t="n">
-        <v>1.116147241011648</v>
-      </c>
-      <c r="J23" s="3" t="n"/>
+        <v>0.7486679427944375</v>
+      </c>
+      <c r="J23" s="3" t="inlineStr">
+        <is>
+          <t>opt_IRR: trial 1602 of kin_opt_ethanol_isobutanol_metabolic_split_12d_pi_log-tail_gp_rb0.001-4_ib0.75-1.5_aA_burden (anchor scenario A; build_opt_IRR_split12d_workbook.py)</t>
+        </is>
+      </c>
       <c r="K23" s="3" t="inlineStr">
         <is>
           <t>V406.nsk_kinetic_model._te.k_1h = x</t>
@@ -1555,7 +1567,11 @@
       <c r="I24" s="3" t="n">
         <v>0.01392</v>
       </c>
-      <c r="J24" s="3" t="n"/>
+      <c r="J24" s="3" t="inlineStr">
+        <is>
+          <t>opt_IRR: trial 1602 of kin_opt_ethanol_isobutanol_metabolic_split_12d_pi_log-tail_gp_rb0.001-4_ib0.75-1.5_aA_burden (anchor scenario A; build_opt_IRR_split12d_workbook.py)</t>
+        </is>
+      </c>
       <c r="K24" s="3" t="inlineStr">
         <is>
           <t>V406.nsk_kinetic_model._te.K_1h = x</t>
@@ -1584,7 +1600,7 @@
         </is>
       </c>
       <c r="E25" s="3" t="n">
-        <v>7.56858807396851</v>
+        <v>50.31715197719465</v>
       </c>
       <c r="F25" s="3" t="inlineStr">
         <is>
@@ -1592,15 +1608,19 @@
         </is>
       </c>
       <c r="G25" s="3" t="n">
-        <v>6.054870459174808</v>
+        <v>40.25372158175572</v>
       </c>
       <c r="H25" s="3" t="n">
-        <v>7.56858807396851</v>
+        <v>50.31715197719465</v>
       </c>
       <c r="I25" s="3" t="n">
-        <v>9.082305688762212</v>
-      </c>
-      <c r="J25" s="3" t="n"/>
+        <v>60.38058237263358</v>
+      </c>
+      <c r="J25" s="3" t="inlineStr">
+        <is>
+          <t>opt_IRR: trial 1602 of kin_opt_ethanol_isobutanol_metabolic_split_12d_pi_log-tail_gp_rb0.001-4_ib0.75-1.5_aA_burden (anchor scenario A; build_opt_IRR_split12d_workbook.py)</t>
+        </is>
+      </c>
       <c r="K25" s="3" t="inlineStr">
         <is>
           <t>V406.nsk_kinetic_model._te.k_1e = x</t>
@@ -1645,7 +1665,11 @@
       <c r="I26" s="3" t="n">
         <v>17.04</v>
       </c>
-      <c r="J26" s="3" t="n"/>
+      <c r="J26" s="3" t="inlineStr">
+        <is>
+          <t>opt_IRR: trial 1602 of kin_opt_ethanol_isobutanol_metabolic_split_12d_pi_log-tail_gp_rb0.001-4_ib0.75-1.5_aA_burden (anchor scenario A; build_opt_IRR_split12d_workbook.py)</t>
+        </is>
+      </c>
       <c r="K26" s="3" t="inlineStr">
         <is>
           <t>V406.nsk_kinetic_model._te.K_1i = x</t>
@@ -1690,7 +1714,11 @@
       <c r="I27" s="3" t="n">
         <v>0.144</v>
       </c>
-      <c r="J27" s="3" t="n"/>
+      <c r="J27" s="3" t="inlineStr">
+        <is>
+          <t>opt_IRR: trial 1602 of kin_opt_ethanol_isobutanol_metabolic_split_12d_pi_log-tail_gp_rb0.001-4_ib0.75-1.5_aA_burden (anchor scenario A; build_opt_IRR_split12d_workbook.py)</t>
+        </is>
+      </c>
       <c r="K27" s="3" t="inlineStr">
         <is>
           <t>V406.nsk_kinetic_model._te.K_1e = x</t>
@@ -1719,7 +1747,7 @@
         </is>
       </c>
       <c r="E28" s="3" t="n">
-        <v>0.004103299498839822</v>
+        <v>0.01618588154641622</v>
       </c>
       <c r="F28" s="3" t="inlineStr">
         <is>
@@ -1727,15 +1755,19 @@
         </is>
       </c>
       <c r="G28" s="3" t="n">
-        <v>0.003282639599071858</v>
+        <v>0.01294870523713298</v>
       </c>
       <c r="H28" s="3" t="n">
-        <v>0.004103299498839822</v>
+        <v>0.01618588154641622</v>
       </c>
       <c r="I28" s="3" t="n">
-        <v>0.004923959398607787</v>
-      </c>
-      <c r="J28" s="3" t="n"/>
+        <v>0.01942305785569947</v>
+      </c>
+      <c r="J28" s="3" t="inlineStr">
+        <is>
+          <t>opt_IRR: trial 1602 of kin_opt_ethanol_isobutanol_metabolic_split_12d_pi_log-tail_gp_rb0.001-4_ib0.75-1.5_aA_burden (anchor scenario A; build_opt_IRR_split12d_workbook.py)</t>
+        </is>
+      </c>
       <c r="K28" s="3" t="inlineStr">
         <is>
           <t>V406.nsk_kinetic_model._te.k_1ie = x</t>
@@ -1764,7 +1796,7 @@
         </is>
       </c>
       <c r="E29" s="3" t="n">
-        <v>0.1051981721819152</v>
+        <v>0.045</v>
       </c>
       <c r="F29" s="3" t="inlineStr">
         <is>
@@ -1772,15 +1804,19 @@
         </is>
       </c>
       <c r="G29" s="3" t="n">
-        <v>0.08415853774553214</v>
+        <v>0.036</v>
       </c>
       <c r="H29" s="3" t="n">
-        <v>0.1051981721819152</v>
+        <v>0.045</v>
       </c>
       <c r="I29" s="3" t="n">
-        <v>0.1262378066182982</v>
-      </c>
-      <c r="J29" s="3" t="n"/>
+        <v>0.054</v>
+      </c>
+      <c r="J29" s="3" t="inlineStr">
+        <is>
+          <t>opt_IRR: trial 1602 of kin_opt_ethanol_isobutanol_metabolic_split_12d_pi_log-tail_gp_rb0.001-4_ib0.75-1.5_aA_burden (anchor scenario A; build_opt_IRR_split12d_workbook.py)</t>
+        </is>
+      </c>
       <c r="K29" s="3" t="inlineStr">
         <is>
           <t>V406.nsk_kinetic_model._te.k_1ia = x</t>
@@ -1809,7 +1845,7 @@
         </is>
       </c>
       <c r="E30" s="3" t="n">
-        <v>0.02027935160978729</v>
+        <v>0.05624999999999999</v>
       </c>
       <c r="F30" s="3" t="inlineStr">
         <is>
@@ -1817,15 +1853,19 @@
         </is>
       </c>
       <c r="G30" s="3" t="n">
-        <v>0.01622348128782984</v>
+        <v>0.045</v>
       </c>
       <c r="H30" s="3" t="n">
-        <v>0.02027935160978729</v>
+        <v>0.05624999999999999</v>
       </c>
       <c r="I30" s="3" t="n">
-        <v>0.02433522193174475</v>
-      </c>
-      <c r="J30" s="3" t="n"/>
+        <v>0.06749999999999999</v>
+      </c>
+      <c r="J30" s="3" t="inlineStr">
+        <is>
+          <t>opt_IRR: trial 1602 of kin_opt_ethanol_isobutanol_metabolic_split_12d_pi_log-tail_gp_rb0.001-4_ib0.75-1.5_aA_burden (anchor scenario A; build_opt_IRR_split12d_workbook.py)</t>
+        </is>
+      </c>
       <c r="K30" s="3" t="inlineStr">
         <is>
           <t>V406.nsk_kinetic_model._te.k_1ii = x</t>
@@ -1870,7 +1910,11 @@
       <c r="I31" s="3" t="n">
         <v>0.6012</v>
       </c>
-      <c r="J31" s="3" t="n"/>
+      <c r="J31" s="3" t="inlineStr">
+        <is>
+          <t>opt_IRR: trial 1602 of kin_opt_ethanol_isobutanol_metabolic_split_12d_pi_log-tail_gp_rb0.001-4_ib0.75-1.5_aA_burden (anchor scenario A; build_opt_IRR_split12d_workbook.py)</t>
+        </is>
+      </c>
       <c r="K31" s="3" t="inlineStr">
         <is>
           <t>V406.nsk_kinetic_model._te.k_2 = x</t>
@@ -1915,7 +1959,11 @@
       <c r="I32" s="3" t="n">
         <v>0.1212</v>
       </c>
-      <c r="J32" s="3" t="n"/>
+      <c r="J32" s="3" t="inlineStr">
+        <is>
+          <t>opt_IRR: trial 1602 of kin_opt_ethanol_isobutanol_metabolic_split_12d_pi_log-tail_gp_rb0.001-4_ib0.75-1.5_aA_burden (anchor scenario A; build_opt_IRR_split12d_workbook.py)</t>
+        </is>
+      </c>
       <c r="K32" s="3" t="inlineStr">
         <is>
           <t>V406.nsk_kinetic_model._te.K_2i = x</t>
@@ -1944,7 +1992,7 @@
         </is>
       </c>
       <c r="E33" s="3" t="n">
-        <v>0.2648468382000104</v>
+        <v>1.278254027285457</v>
       </c>
       <c r="F33" s="3" t="inlineStr">
         <is>
@@ -1952,15 +2000,19 @@
         </is>
       </c>
       <c r="G33" s="3" t="n">
-        <v>0.2118774705600083</v>
+        <v>1.022603221828366</v>
       </c>
       <c r="H33" s="3" t="n">
-        <v>0.2648468382000104</v>
+        <v>1.278254027285457</v>
       </c>
       <c r="I33" s="3" t="n">
-        <v>0.3178162058400124</v>
-      </c>
-      <c r="J33" s="3" t="n"/>
+        <v>1.533904832742549</v>
+      </c>
+      <c r="J33" s="3" t="inlineStr">
+        <is>
+          <t>opt_IRR: trial 1602 of kin_opt_ethanol_isobutanol_metabolic_split_12d_pi_log-tail_gp_rb0.001-4_ib0.75-1.5_aA_burden (anchor scenario A; build_opt_IRR_split12d_workbook.py)</t>
+        </is>
+      </c>
       <c r="K33" s="3" t="inlineStr">
         <is>
           <t>V406.nsk_kinetic_model._te.k_3 = x</t>
@@ -2005,7 +2057,11 @@
       <c r="I34" s="5" t="n">
         <v>6e-07</v>
       </c>
-      <c r="J34" s="3" t="n"/>
+      <c r="J34" s="3" t="inlineStr">
+        <is>
+          <t>opt_IRR: trial 1602 of kin_opt_ethanol_isobutanol_metabolic_split_12d_pi_log-tail_gp_rb0.001-4_ib0.75-1.5_aA_burden (anchor scenario A; build_opt_IRR_split12d_workbook.py)</t>
+        </is>
+      </c>
       <c r="K34" s="3" t="inlineStr">
         <is>
           <t>V406.nsk_kinetic_model._te.K_3 = x</t>
@@ -2050,7 +2106,11 @@
       <c r="I35" s="3" t="n">
         <v>5.76</v>
       </c>
-      <c r="J35" s="3" t="n"/>
+      <c r="J35" s="3" t="inlineStr">
+        <is>
+          <t>opt_IRR: trial 1602 of kin_opt_ethanol_isobutanol_metabolic_split_12d_pi_log-tail_gp_rb0.001-4_ib0.75-1.5_aA_burden (anchor scenario A; build_opt_IRR_split12d_workbook.py)</t>
+        </is>
+      </c>
       <c r="K35" s="3" t="inlineStr">
         <is>
           <t>V406.nsk_kinetic_model._te.k_4 = x</t>
@@ -2079,7 +2139,7 @@
         </is>
       </c>
       <c r="E36" s="3" t="n">
-        <v>0.008206598997679644</v>
+        <v>0.03237176309283245</v>
       </c>
       <c r="F36" s="3" t="inlineStr">
         <is>
@@ -2087,15 +2147,19 @@
         </is>
       </c>
       <c r="G36" s="3" t="n">
-        <v>0.006565279198143716</v>
+        <v>0.02589741047426596</v>
       </c>
       <c r="H36" s="3" t="n">
-        <v>0.008206598997679644</v>
+        <v>0.03237176309283245</v>
       </c>
       <c r="I36" s="3" t="n">
-        <v>0.009847918797215574</v>
-      </c>
-      <c r="J36" s="3" t="n"/>
+        <v>0.03884611571139893</v>
+      </c>
+      <c r="J36" s="3" t="inlineStr">
+        <is>
+          <t>opt_IRR: trial 1602 of kin_opt_ethanol_isobutanol_metabolic_split_12d_pi_log-tail_gp_rb0.001-4_ib0.75-1.5_aA_burden (anchor scenario A; build_opt_IRR_split12d_workbook.py)</t>
+        </is>
+      </c>
       <c r="K36" s="3" t="inlineStr">
         <is>
           <t>V406.nsk_kinetic_model._te.k_4ie = x</t>
@@ -2124,7 +2188,7 @@
         </is>
       </c>
       <c r="E37" s="3" t="n">
-        <v>0.2103963443638303</v>
+        <v>0.09</v>
       </c>
       <c r="F37" s="3" t="inlineStr">
         <is>
@@ -2132,15 +2196,19 @@
         </is>
       </c>
       <c r="G37" s="3" t="n">
-        <v>0.1683170754910643</v>
+        <v>0.07199999999999999</v>
       </c>
       <c r="H37" s="3" t="n">
-        <v>0.2103963443638303</v>
+        <v>0.09</v>
       </c>
       <c r="I37" s="3" t="n">
-        <v>0.2524756132365964</v>
-      </c>
-      <c r="J37" s="3" t="n"/>
+        <v>0.108</v>
+      </c>
+      <c r="J37" s="3" t="inlineStr">
+        <is>
+          <t>opt_IRR: trial 1602 of kin_opt_ethanol_isobutanol_metabolic_split_12d_pi_log-tail_gp_rb0.001-4_ib0.75-1.5_aA_burden (anchor scenario A; build_opt_IRR_split12d_workbook.py)</t>
+        </is>
+      </c>
       <c r="K37" s="3" t="inlineStr">
         <is>
           <t>V406.nsk_kinetic_model._te.k_4ia = x</t>
@@ -2169,7 +2237,7 @@
         </is>
       </c>
       <c r="E38" s="3" t="n">
-        <v>0.04055870321957459</v>
+        <v>0.1125</v>
       </c>
       <c r="F38" s="3" t="inlineStr">
         <is>
@@ -2177,15 +2245,19 @@
         </is>
       </c>
       <c r="G38" s="3" t="n">
-        <v>0.03244696257565968</v>
+        <v>0.09</v>
       </c>
       <c r="H38" s="3" t="n">
-        <v>0.04055870321957459</v>
+        <v>0.1125</v>
       </c>
       <c r="I38" s="3" t="n">
-        <v>0.0486704438634895</v>
-      </c>
-      <c r="J38" s="3" t="n"/>
+        <v>0.135</v>
+      </c>
+      <c r="J38" s="3" t="inlineStr">
+        <is>
+          <t>opt_IRR: trial 1602 of kin_opt_ethanol_isobutanol_metabolic_split_12d_pi_log-tail_gp_rb0.001-4_ib0.75-1.5_aA_burden (anchor scenario A; build_opt_IRR_split12d_workbook.py)</t>
+        </is>
+      </c>
       <c r="K38" s="3" t="inlineStr">
         <is>
           <t>V406.nsk_kinetic_model._te.k_4ii = x</t>
@@ -2230,7 +2302,11 @@
       <c r="I39" s="3" t="n">
         <v>0.0003168</v>
       </c>
-      <c r="J39" s="3" t="n"/>
+      <c r="J39" s="3" t="inlineStr">
+        <is>
+          <t>opt_IRR: trial 1602 of kin_opt_ethanol_isobutanol_metabolic_split_12d_pi_log-tail_gp_rb0.001-4_ib0.75-1.5_aA_burden (anchor scenario A; build_opt_IRR_split12d_workbook.py)</t>
+        </is>
+      </c>
       <c r="K39" s="3" t="inlineStr">
         <is>
           <t>V406.nsk_kinetic_model._te.K_4 = x</t>
@@ -2275,7 +2351,11 @@
       <c r="I40" s="3" t="n">
         <v>0.01248</v>
       </c>
-      <c r="J40" s="3" t="n"/>
+      <c r="J40" s="3" t="inlineStr">
+        <is>
+          <t>opt_IRR: trial 1602 of kin_opt_ethanol_isobutanol_metabolic_split_12d_pi_log-tail_gp_rb0.001-4_ib0.75-1.5_aA_burden (anchor scenario A; build_opt_IRR_split12d_workbook.py)</t>
+        </is>
+      </c>
       <c r="K40" s="3" t="inlineStr">
         <is>
           <t>V406.nsk_kinetic_model._te.k_5 = x</t>
@@ -2320,7 +2400,11 @@
       <c r="I41" s="3" t="n">
         <v>0.01224</v>
       </c>
-      <c r="J41" s="3" t="n"/>
+      <c r="J41" s="3" t="inlineStr">
+        <is>
+          <t>opt_IRR: trial 1602 of kin_opt_ethanol_isobutanol_metabolic_split_12d_pi_log-tail_gp_rb0.001-4_ib0.75-1.5_aA_burden (anchor scenario A; build_opt_IRR_split12d_workbook.py)</t>
+        </is>
+      </c>
       <c r="K41" s="3" t="inlineStr">
         <is>
           <t>V406.nsk_kinetic_model._te.K_5 = x</t>
@@ -2365,7 +2449,11 @@
       <c r="I42" s="3" t="n">
         <v>0.9299999999999999</v>
       </c>
-      <c r="J42" s="3" t="n"/>
+      <c r="J42" s="3" t="inlineStr">
+        <is>
+          <t>opt_IRR: trial 1602 of kin_opt_ethanol_isobutanol_metabolic_split_12d_pi_log-tail_gp_rb0.001-4_ib0.75-1.5_aA_burden (anchor scenario A; build_opt_IRR_split12d_workbook.py)</t>
+        </is>
+      </c>
       <c r="K42" s="3" t="inlineStr">
         <is>
           <t>V406.nsk_kinetic_model._te.k_5e = x</t>
@@ -2410,7 +2498,11 @@
       <c r="I43" s="3" t="n">
         <v>0.12</v>
       </c>
-      <c r="J43" s="3" t="n"/>
+      <c r="J43" s="3" t="inlineStr">
+        <is>
+          <t>opt_IRR: trial 1602 of kin_opt_ethanol_isobutanol_metabolic_split_12d_pi_log-tail_gp_rb0.001-4_ib0.75-1.5_aA_burden (anchor scenario A; build_opt_IRR_split12d_workbook.py)</t>
+        </is>
+      </c>
       <c r="K43" s="3" t="inlineStr">
         <is>
           <t>V406.nsk_kinetic_model._te.K_5e = x</t>
@@ -2455,7 +2547,11 @@
       <c r="I44" s="3" t="n">
         <v>528</v>
       </c>
-      <c r="J44" s="3" t="n"/>
+      <c r="J44" s="3" t="inlineStr">
+        <is>
+          <t>opt_IRR: trial 1602 of kin_opt_ethanol_isobutanol_metabolic_split_12d_pi_log-tail_gp_rb0.001-4_ib0.75-1.5_aA_burden (anchor scenario A; build_opt_IRR_split12d_workbook.py)</t>
+        </is>
+      </c>
       <c r="K44" s="3" t="inlineStr">
         <is>
           <t>V406.nsk_kinetic_model._te.K_5i = x</t>
@@ -2484,7 +2580,7 @@
         </is>
       </c>
       <c r="E45" s="3" t="n">
-        <v>23.48573338352841</v>
+        <v>2.199496289405869</v>
       </c>
       <c r="F45" s="3" t="inlineStr">
         <is>
@@ -2492,15 +2588,19 @@
         </is>
       </c>
       <c r="G45" s="3" t="n">
-        <v>18.78858670682272</v>
+        <v>1.759597031524696</v>
       </c>
       <c r="H45" s="3" t="n">
-        <v>23.48573338352841</v>
+        <v>2.199496289405869</v>
       </c>
       <c r="I45" s="3" t="n">
-        <v>28.18288006023409</v>
-      </c>
-      <c r="J45" s="3" t="n"/>
+        <v>2.639395547287043</v>
+      </c>
+      <c r="J45" s="3" t="inlineStr">
+        <is>
+          <t>opt_IRR: trial 1602 of kin_opt_ethanol_isobutanol_metabolic_split_12d_pi_log-tail_gp_rb0.001-4_ib0.75-1.5_aA_burden (anchor scenario A; build_opt_IRR_split12d_workbook.py)</t>
+        </is>
+      </c>
       <c r="K45" s="3" t="inlineStr">
         <is>
           <t>V406.nsk_kinetic_model._te.k_6 = x</t>
@@ -2545,7 +2645,11 @@
       <c r="I46" s="3" t="n">
         <v>0.0408</v>
       </c>
-      <c r="J46" s="3" t="n"/>
+      <c r="J46" s="3" t="inlineStr">
+        <is>
+          <t>opt_IRR: trial 1602 of kin_opt_ethanol_isobutanol_metabolic_split_12d_pi_log-tail_gp_rb0.001-4_ib0.75-1.5_aA_burden (anchor scenario A; build_opt_IRR_split12d_workbook.py)</t>
+        </is>
+      </c>
       <c r="K46" s="3" t="inlineStr">
         <is>
           <t>V406.nsk_kinetic_model._te.K_6 = x</t>
@@ -2590,7 +2694,11 @@
       <c r="I47" s="3" t="n">
         <v>0.0684</v>
       </c>
-      <c r="J47" s="3" t="n"/>
+      <c r="J47" s="3" t="inlineStr">
+        <is>
+          <t>opt_IRR: trial 1602 of kin_opt_ethanol_isobutanol_metabolic_split_12d_pi_log-tail_gp_rb0.001-4_ib0.75-1.5_aA_burden (anchor scenario A; build_opt_IRR_split12d_workbook.py)</t>
+        </is>
+      </c>
       <c r="K47" s="3" t="inlineStr">
         <is>
           <t>V406.nsk_kinetic_model._te.K_6e = x</t>
@@ -2619,7 +2727,7 @@
         </is>
       </c>
       <c r="E48" t="n">
-        <v>0.1051981721819152</v>
+        <v>0.045</v>
       </c>
       <c r="F48" t="inlineStr">
         <is>
@@ -2627,13 +2735,18 @@
         </is>
       </c>
       <c r="G48" t="n">
-        <v>0.08415853774553214</v>
+        <v>0.036</v>
       </c>
       <c r="H48" t="n">
-        <v>0.1051981721819152</v>
+        <v>0.045</v>
       </c>
       <c r="I48" t="n">
-        <v>0.1262378066182982</v>
+        <v>0.054</v>
+      </c>
+      <c r="J48" t="inlineStr">
+        <is>
+          <t>opt_IRR: trial 1602 of kin_opt_ethanol_isobutanol_metabolic_split_12d_pi_log-tail_gp_rb0.001-4_ib0.75-1.5_aA_burden (anchor scenario A; build_opt_IRR_split12d_workbook.py)</t>
+        </is>
       </c>
       <c r="K48" t="inlineStr">
         <is>
@@ -2663,7 +2776,7 @@
         </is>
       </c>
       <c r="E49" t="n">
-        <v>0.02027935160978729</v>
+        <v>0.05624999999999999</v>
       </c>
       <c r="F49" t="inlineStr">
         <is>
@@ -2671,13 +2784,18 @@
         </is>
       </c>
       <c r="G49" t="n">
-        <v>0.01622348128782984</v>
+        <v>0.045</v>
       </c>
       <c r="H49" t="n">
-        <v>0.02027935160978729</v>
+        <v>0.05624999999999999</v>
       </c>
       <c r="I49" t="n">
-        <v>0.02433522193174475</v>
+        <v>0.06749999999999999</v>
+      </c>
+      <c r="J49" t="inlineStr">
+        <is>
+          <t>opt_IRR: trial 1602 of kin_opt_ethanol_isobutanol_metabolic_split_12d_pi_log-tail_gp_rb0.001-4_ib0.75-1.5_aA_burden (anchor scenario A; build_opt_IRR_split12d_workbook.py)</t>
+        </is>
       </c>
       <c r="K49" t="inlineStr">
         <is>
@@ -2723,7 +2841,11 @@
       <c r="I50" s="3" t="n">
         <v>1.4436</v>
       </c>
-      <c r="J50" s="3" t="n"/>
+      <c r="J50" s="3" t="inlineStr">
+        <is>
+          <t>opt_IRR: trial 1602 of kin_opt_ethanol_isobutanol_metabolic_split_12d_pi_log-tail_gp_rb0.001-4_ib0.75-1.5_aA_burden (anchor scenario A; build_opt_IRR_split12d_workbook.py)</t>
+        </is>
+      </c>
       <c r="K50" s="3" t="inlineStr">
         <is>
           <t>V406.nsk_kinetic_model._te.k_7 = x</t>
@@ -2752,7 +2874,7 @@
         </is>
       </c>
       <c r="E51" s="3" t="n">
-        <v>0.008206598997679644</v>
+        <v>0.03237176309283245</v>
       </c>
       <c r="F51" s="3" t="inlineStr">
         <is>
@@ -2760,15 +2882,19 @@
         </is>
       </c>
       <c r="G51" s="3" t="n">
-        <v>0.006565279198143716</v>
+        <v>0.02589741047426596</v>
       </c>
       <c r="H51" s="3" t="n">
-        <v>0.008206598997679644</v>
+        <v>0.03237176309283245</v>
       </c>
       <c r="I51" s="3" t="n">
-        <v>0.009847918797215574</v>
-      </c>
-      <c r="J51" s="3" t="n"/>
+        <v>0.03884611571139893</v>
+      </c>
+      <c r="J51" s="3" t="inlineStr">
+        <is>
+          <t>opt_IRR: trial 1602 of kin_opt_ethanol_isobutanol_metabolic_split_12d_pi_log-tail_gp_rb0.001-4_ib0.75-1.5_aA_burden (anchor scenario A; build_opt_IRR_split12d_workbook.py)</t>
+        </is>
+      </c>
       <c r="K51" s="3" t="inlineStr">
         <is>
           <t>V406.nsk_kinetic_model._te.k_7ie = x</t>
@@ -2797,7 +2923,7 @@
         </is>
       </c>
       <c r="E52" s="3" t="n">
-        <v>0.2103963443638303</v>
+        <v>0.09</v>
       </c>
       <c r="F52" s="3" t="inlineStr">
         <is>
@@ -2805,15 +2931,19 @@
         </is>
       </c>
       <c r="G52" s="3" t="n">
-        <v>0.1683170754910643</v>
+        <v>0.07199999999999999</v>
       </c>
       <c r="H52" s="3" t="n">
-        <v>0.2103963443638303</v>
+        <v>0.09</v>
       </c>
       <c r="I52" s="3" t="n">
-        <v>0.2524756132365964</v>
-      </c>
-      <c r="J52" s="3" t="n"/>
+        <v>0.108</v>
+      </c>
+      <c r="J52" s="3" t="inlineStr">
+        <is>
+          <t>opt_IRR: trial 1602 of kin_opt_ethanol_isobutanol_metabolic_split_12d_pi_log-tail_gp_rb0.001-4_ib0.75-1.5_aA_burden (anchor scenario A; build_opt_IRR_split12d_workbook.py)</t>
+        </is>
+      </c>
       <c r="K52" s="3" t="inlineStr">
         <is>
           <t>V406.nsk_kinetic_model._te.k_7ia = x</t>
@@ -2842,7 +2972,7 @@
         </is>
       </c>
       <c r="E53" s="3" t="n">
-        <v>0.04055870321957459</v>
+        <v>0.1125</v>
       </c>
       <c r="F53" s="3" t="inlineStr">
         <is>
@@ -2850,15 +2980,19 @@
         </is>
       </c>
       <c r="G53" s="3" t="n">
-        <v>0.03244696257565968</v>
+        <v>0.09</v>
       </c>
       <c r="H53" s="3" t="n">
-        <v>0.04055870321957459</v>
+        <v>0.1125</v>
       </c>
       <c r="I53" s="3" t="n">
-        <v>0.0486704438634895</v>
-      </c>
-      <c r="J53" s="3" t="n"/>
+        <v>0.135</v>
+      </c>
+      <c r="J53" s="3" t="inlineStr">
+        <is>
+          <t>opt_IRR: trial 1602 of kin_opt_ethanol_isobutanol_metabolic_split_12d_pi_log-tail_gp_rb0.001-4_ib0.75-1.5_aA_burden (anchor scenario A; build_opt_IRR_split12d_workbook.py)</t>
+        </is>
+      </c>
       <c r="K53" s="3" t="inlineStr">
         <is>
           <t>V406.nsk_kinetic_model._te.k_7ii = x</t>
@@ -2903,7 +3037,11 @@
       <c r="I54" s="3" t="n">
         <v>0.01212</v>
       </c>
-      <c r="J54" s="3" t="n"/>
+      <c r="J54" s="3" t="inlineStr">
+        <is>
+          <t>opt_IRR: trial 1602 of kin_opt_ethanol_isobutanol_metabolic_split_12d_pi_log-tail_gp_rb0.001-4_ib0.75-1.5_aA_burden (anchor scenario A; build_opt_IRR_split12d_workbook.py)</t>
+        </is>
+      </c>
       <c r="K54" s="3" t="inlineStr">
         <is>
           <t>V406.nsk_kinetic_model._te.K_7 = x</t>
@@ -2948,7 +3086,11 @@
       <c r="I55" s="3" t="n">
         <v>0.7068</v>
       </c>
-      <c r="J55" s="3" t="n"/>
+      <c r="J55" s="3" t="inlineStr">
+        <is>
+          <t>opt_IRR: trial 1602 of kin_opt_ethanol_isobutanol_metabolic_split_12d_pi_log-tail_gp_rb0.001-4_ib0.75-1.5_aA_burden (anchor scenario A; build_opt_IRR_split12d_workbook.py)</t>
+        </is>
+      </c>
       <c r="K55" s="3" t="inlineStr">
         <is>
           <t>V406.nsk_kinetic_model._te.k_8 = x</t>
@@ -2993,7 +3135,11 @@
       <c r="I56" s="3" t="n">
         <v>0.009599999999999999</v>
       </c>
-      <c r="J56" s="3" t="n"/>
+      <c r="J56" s="3" t="inlineStr">
+        <is>
+          <t>opt_IRR: trial 1602 of kin_opt_ethanol_isobutanol_metabolic_split_12d_pi_log-tail_gp_rb0.001-4_ib0.75-1.5_aA_burden (anchor scenario A; build_opt_IRR_split12d_workbook.py)</t>
+        </is>
+      </c>
       <c r="K56" s="3" t="inlineStr">
         <is>
           <t>V406.nsk_kinetic_model._te.k_9 = x</t>
@@ -3038,7 +3184,11 @@
       <c r="I57" s="3" t="n">
         <v>0.09011999999999999</v>
       </c>
-      <c r="J57" s="3" t="n"/>
+      <c r="J57" s="3" t="inlineStr">
+        <is>
+          <t>opt_IRR: trial 1602 of kin_opt_ethanol_isobutanol_metabolic_split_12d_pi_log-tail_gp_rb0.001-4_ib0.75-1.5_aA_burden (anchor scenario A; build_opt_IRR_split12d_workbook.py)</t>
+        </is>
+      </c>
       <c r="K57" s="3" t="inlineStr">
         <is>
           <t>V406.nsk_kinetic_model._te.k_9e = x</t>
@@ -3083,7 +3233,11 @@
       <c r="I58" s="3" t="n">
         <v>15.6</v>
       </c>
-      <c r="J58" s="3" t="n"/>
+      <c r="J58" s="3" t="inlineStr">
+        <is>
+          <t>opt_IRR: trial 1602 of kin_opt_ethanol_isobutanol_metabolic_split_12d_pi_log-tail_gp_rb0.001-4_ib0.75-1.5_aA_burden (anchor scenario A; build_opt_IRR_split12d_workbook.py)</t>
+        </is>
+      </c>
       <c r="K58" s="3" t="inlineStr">
         <is>
           <t>V406.nsk_kinetic_model._te.K_9e = x</t>
@@ -3128,7 +3282,11 @@
       <c r="I59" s="3" t="n">
         <v>30</v>
       </c>
-      <c r="J59" s="3" t="n"/>
+      <c r="J59" s="3" t="inlineStr">
+        <is>
+          <t>opt_IRR: trial 1602 of kin_opt_ethanol_isobutanol_metabolic_split_12d_pi_log-tail_gp_rb0.001-4_ib0.75-1.5_aA_burden (anchor scenario A; build_opt_IRR_split12d_workbook.py)</t>
+        </is>
+      </c>
       <c r="K59" s="3" t="inlineStr">
         <is>
           <t>V406.nsk_kinetic_model._te.K_9i = x</t>
@@ -3173,7 +3331,11 @@
       <c r="I60" s="3" t="n">
         <v>0.004788</v>
       </c>
-      <c r="J60" s="3" t="n"/>
+      <c r="J60" s="3" t="inlineStr">
+        <is>
+          <t>opt_IRR: trial 1602 of kin_opt_ethanol_isobutanol_metabolic_split_12d_pi_log-tail_gp_rb0.001-4_ib0.75-1.5_aA_burden (anchor scenario A; build_opt_IRR_split12d_workbook.py)</t>
+        </is>
+      </c>
       <c r="K60" s="3" t="inlineStr">
         <is>
           <t>V406.nsk_kinetic_model._te.k_9c = x</t>
@@ -3218,7 +3380,11 @@
       <c r="I61" s="3" t="n">
         <v>0.07199999999999999</v>
       </c>
-      <c r="J61" s="3" t="n"/>
+      <c r="J61" s="3" t="inlineStr">
+        <is>
+          <t>opt_IRR: trial 1602 of kin_opt_ethanol_isobutanol_metabolic_split_12d_pi_log-tail_gp_rb0.001-4_ib0.75-1.5_aA_burden (anchor scenario A; build_opt_IRR_split12d_workbook.py)</t>
+        </is>
+      </c>
       <c r="K61" s="3" t="inlineStr">
         <is>
           <t>V406.nsk_kinetic_model._te.k_10 = x</t>
@@ -3247,7 +3413,7 @@
         </is>
       </c>
       <c r="E62" t="n">
-        <v>0.008206598997679644</v>
+        <v>0.03237176309283245</v>
       </c>
       <c r="F62" t="inlineStr">
         <is>
@@ -3255,13 +3421,18 @@
         </is>
       </c>
       <c r="G62" t="n">
-        <v>0.006565279198143716</v>
+        <v>0.02589741047426596</v>
       </c>
       <c r="H62" t="n">
-        <v>0.008206598997679644</v>
+        <v>0.03237176309283245</v>
       </c>
       <c r="I62" t="n">
-        <v>0.009847918797215574</v>
+        <v>0.03884611571139893</v>
+      </c>
+      <c r="J62" t="inlineStr">
+        <is>
+          <t>opt_IRR: trial 1602 of kin_opt_ethanol_isobutanol_metabolic_split_12d_pi_log-tail_gp_rb0.001-4_ib0.75-1.5_aA_burden (anchor scenario A; build_opt_IRR_split12d_workbook.py)</t>
+        </is>
       </c>
       <c r="K62" t="inlineStr">
         <is>
@@ -3291,7 +3462,7 @@
         </is>
       </c>
       <c r="E63" t="n">
-        <v>0.2103963443638303</v>
+        <v>0.09</v>
       </c>
       <c r="F63" t="inlineStr">
         <is>
@@ -3299,13 +3470,18 @@
         </is>
       </c>
       <c r="G63" t="n">
-        <v>0.1683170754910643</v>
+        <v>0.07199999999999999</v>
       </c>
       <c r="H63" t="n">
-        <v>0.2103963443638303</v>
+        <v>0.09</v>
       </c>
       <c r="I63" t="n">
-        <v>0.2524756132365964</v>
+        <v>0.108</v>
+      </c>
+      <c r="J63" t="inlineStr">
+        <is>
+          <t>opt_IRR: trial 1602 of kin_opt_ethanol_isobutanol_metabolic_split_12d_pi_log-tail_gp_rb0.001-4_ib0.75-1.5_aA_burden (anchor scenario A; build_opt_IRR_split12d_workbook.py)</t>
+        </is>
       </c>
       <c r="K63" t="inlineStr">
         <is>
@@ -3335,7 +3511,7 @@
         </is>
       </c>
       <c r="E64" t="n">
-        <v>0.04055870321957459</v>
+        <v>0.1125</v>
       </c>
       <c r="F64" t="inlineStr">
         <is>
@@ -3343,13 +3519,18 @@
         </is>
       </c>
       <c r="G64" t="n">
-        <v>0.03244696257565968</v>
+        <v>0.09</v>
       </c>
       <c r="H64" t="n">
-        <v>0.04055870321957459</v>
+        <v>0.1125</v>
       </c>
       <c r="I64" t="n">
-        <v>0.0486704438634895</v>
+        <v>0.135</v>
+      </c>
+      <c r="J64" t="inlineStr">
+        <is>
+          <t>opt_IRR: trial 1602 of kin_opt_ethanol_isobutanol_metabolic_split_12d_pi_log-tail_gp_rb0.001-4_ib0.75-1.5_aA_burden (anchor scenario A; build_opt_IRR_split12d_workbook.py)</t>
+        </is>
       </c>
       <c r="K64" t="inlineStr">
         <is>
@@ -3395,7 +3576,11 @@
       <c r="I65" s="3" t="n">
         <v>0.024</v>
       </c>
-      <c r="J65" s="3" t="n"/>
+      <c r="J65" s="3" t="inlineStr">
+        <is>
+          <t>opt_IRR: trial 1602 of kin_opt_ethanol_isobutanol_metabolic_split_12d_pi_log-tail_gp_rb0.001-4_ib0.75-1.5_aA_burden (anchor scenario A; build_opt_IRR_split12d_workbook.py)</t>
+        </is>
+      </c>
       <c r="K65" s="3" t="inlineStr">
         <is>
           <t>V406.nsk_kinetic_model._te.k_11 = x</t>
@@ -3424,7 +3609,7 @@
         </is>
       </c>
       <c r="E66" s="3" t="n">
-        <v>0.6421409697576548</v>
+        <v>4</v>
       </c>
       <c r="F66" s="3" t="inlineStr">
         <is>
@@ -3432,15 +3617,19 @@
         </is>
       </c>
       <c r="G66" s="5" t="n">
-        <v>0.5137127758061238</v>
+        <v>3.2</v>
       </c>
       <c r="H66" s="5" t="n">
-        <v>0.6421409697576548</v>
+        <v>4</v>
       </c>
       <c r="I66" s="5" t="n">
-        <v>0.7705691637091857</v>
-      </c>
-      <c r="J66" s="3" t="n"/>
+        <v>4.8</v>
+      </c>
+      <c r="J66" s="3" t="inlineStr">
+        <is>
+          <t>opt_IRR: trial 1602 of kin_opt_ethanol_isobutanol_metabolic_split_12d_pi_log-tail_gp_rb0.001-4_ib0.75-1.5_aA_burden (anchor scenario A; build_opt_IRR_split12d_workbook.py)</t>
+        </is>
+      </c>
       <c r="K66" s="3" t="inlineStr">
         <is>
           <t>V406.nsk_kinetic_model._te.k_13 = x</t>
@@ -3477,7 +3666,7 @@
         </is>
       </c>
       <c r="G67" s="5" t="n">
-        <v>0.08</v>
+        <v>0.08000000000000002</v>
       </c>
       <c r="H67" s="5" t="n">
         <v>0.1</v>
@@ -3487,7 +3676,7 @@
       </c>
       <c r="J67" s="3" t="inlineStr">
         <is>
-          <t>K_13 = 0.10 g/L: ALS/Pdc pyruvate-affinity ratio (Ilv2/Ilv6 Km 3.9 mM, BRENDA EC 2.2.1.6; Pang &amp; Duggleby 1999 doi:10.1021/bi983013m; Pdc wild-type Km 0.5-1.1 mM, BRENDA EC 4.1.1.1) x r3 half-saturation 0.027 g/L; r13 is Michaelis-Menten since 2026-09-13 (was 5e-7, copied from K_3). +-20% kinetic convention. See docs/reports/r13-rate-law.md</t>
+          <t>opt_IRR: trial 1602 of kin_opt_ethanol_isobutanol_metabolic_split_12d_pi_log-tail_gp_rb0.001-4_ib0.75-1.5_aA_burden (anchor scenario A; build_opt_IRR_split12d_workbook.py) | template note: K_13 = 0.10 g/L: ALS/Pdc pyruvate-affinity ratio (Ilv2/Ilv6 Km 3.9 mM, BRENDA EC 2.2.1.6; Pang &amp; Duggleby 1999 doi:10.1021/bi983013m; Pdc wild-type Km 0.5-1.1 mM, BRENDA EC 4.1.1.1) x r3 half-saturation 0.027 g/L; r13 is Michaelis-Menten since 2026-09-13 (was 5e-7, copied from K_3). +-20% kinetic convention. See docs/reports/r13-rate-law.md</t>
         </is>
       </c>
       <c r="K67" s="3" t="inlineStr">
@@ -3518,7 +3707,7 @@
         </is>
       </c>
       <c r="E68" s="3" t="n">
-        <v>0.6228252477025641</v>
+        <v>0.8131870187402369</v>
       </c>
       <c r="F68" s="3" t="inlineStr">
         <is>
@@ -3526,15 +3715,19 @@
         </is>
       </c>
       <c r="G68" s="5" t="n">
-        <v>0.4982601981620513</v>
+        <v>0.6505496149921896</v>
       </c>
       <c r="H68" s="5" t="n">
-        <v>0.6228252477025641</v>
+        <v>0.8131870187402369</v>
       </c>
       <c r="I68" s="5" t="n">
-        <v>0.7473902972430769</v>
-      </c>
-      <c r="J68" s="3" t="n"/>
+        <v>0.9758244224882843</v>
+      </c>
+      <c r="J68" s="3" t="inlineStr">
+        <is>
+          <t>opt_IRR: trial 1602 of kin_opt_ethanol_isobutanol_metabolic_split_12d_pi_log-tail_gp_rb0.001-4_ib0.75-1.5_aA_burden (anchor scenario A; build_opt_IRR_split12d_workbook.py)</t>
+        </is>
+      </c>
       <c r="K68" s="3" t="inlineStr">
         <is>
           <t>V406.nsk_kinetic_model._te.k_14 = x</t>
@@ -3581,7 +3774,7 @@
       </c>
       <c r="J69" s="3" t="inlineStr">
         <is>
-          <t>K_14 = 0.017 g/L: KARI (Ilv5) acetolactate affinity. N. crassa reductoisomerase surrogate Km 0.32 mM (Kiritani et al. 1966 JBC 241:2047; BRENDA EC 1.1.1.86) = 0.042 g/L acetolactate (132.11 g/mol) x in-vivo/in-vitro scale factor S = 0.4 read off Lei's fitted r3/r4/r6 constants (S = 0.27-0.60 / 0.17-0.25 / 0.70). nskinetics b61360e, 2026-09-13 (was 2.64e-4, copied from K_4). +-20% kinetic convention (band over the S range 0.007-0.030 is for a dedicated sweep only). See nskinetics docs/reports/r14-r16-rate-laws-and-affinity-anchoring.md (2026-09-13).</t>
+          <t>opt_IRR: trial 1602 of kin_opt_ethanol_isobutanol_metabolic_split_12d_pi_log-tail_gp_rb0.001-4_ib0.75-1.5_aA_burden (anchor scenario A; build_opt_IRR_split12d_workbook.py) | template note: K_14 = 0.017 g/L: KARI (Ilv5) acetolactate affinity. N. crassa reductoisomerase surrogate Km 0.32 mM (Kiritani et al. 1966 JBC 241:2047; BRENDA EC 1.1.1.86) = 0.042 g/L acetolactate (132.11 g/mol) x in-vivo/in-vitro scale factor S = 0.4 read off Lei's fitted r3/r4/r6 constants (S = 0.27-0.60 / 0.17-0.25 / 0.70). nskinetics b61360e, 2026-09-13 (was 2.64e-4, copied from K_4). +-20% kinetic convention (band over the S range 0.007-0.030 is for a dedicated sweep only). See nskinetics docs/reports/r14-r16-rate-laws-and-affinity-anchoring.md (2026-09-13).</t>
         </is>
       </c>
       <c r="K69" s="3" t="inlineStr">
@@ -3612,7 +3805,7 @@
         </is>
       </c>
       <c r="E70" s="3" t="n">
-        <v>0.4590182352522549</v>
+        <v>0.8253848240213404</v>
       </c>
       <c r="F70" s="3" t="inlineStr">
         <is>
@@ -3620,15 +3813,19 @@
         </is>
       </c>
       <c r="G70" s="5" t="n">
-        <v>0.3672145882018039</v>
+        <v>0.6603078592170724</v>
       </c>
       <c r="H70" s="5" t="n">
-        <v>0.4590182352522549</v>
+        <v>0.8253848240213404</v>
       </c>
       <c r="I70" s="5" t="n">
-        <v>0.5508218823027058</v>
-      </c>
-      <c r="J70" s="3" t="n"/>
+        <v>0.9904617888256084</v>
+      </c>
+      <c r="J70" s="3" t="inlineStr">
+        <is>
+          <t>opt_IRR: trial 1602 of kin_opt_ethanol_isobutanol_metabolic_split_12d_pi_log-tail_gp_rb0.001-4_ib0.75-1.5_aA_burden (anchor scenario A; build_opt_IRR_split12d_workbook.py)</t>
+        </is>
+      </c>
       <c r="K70" s="3" t="inlineStr">
         <is>
           <t>V406.nsk_kinetic_model._te.k_15 = x</t>
@@ -3675,7 +3872,7 @@
       </c>
       <c r="J71" s="3" t="inlineStr">
         <is>
-          <t>K_15 = 0.080 g/L: DHAD (Ilv3) DHIV affinity. E. coli IlvD surrogate Km 1.5 mM (Flint et al. 1993 JBC 268:14732; BRENDA EC 4.2.1.9) = 0.201 g/L DHIV (134.13 g/mol) x S = 0.4. nskinetics b61360e, 2026-09-13 (was 2.64e-4, copied from K_4). +-20% kinetic convention (band over the S range 0.034-0.14 is for a dedicated sweep only). See nskinetics docs/reports/r14-r16-rate-laws-and-affinity-anchoring.md (2026-09-13).</t>
+          <t>opt_IRR: trial 1602 of kin_opt_ethanol_isobutanol_metabolic_split_12d_pi_log-tail_gp_rb0.001-4_ib0.75-1.5_aA_burden (anchor scenario A; build_opt_IRR_split12d_workbook.py) | template note: K_15 = 0.080 g/L: DHAD (Ilv3) DHIV affinity. E. coli IlvD surrogate Km 1.5 mM (Flint et al. 1993 JBC 268:14732; BRENDA EC 4.2.1.9) = 0.201 g/L DHIV (134.13 g/mol) x S = 0.4. nskinetics b61360e, 2026-09-13 (was 2.64e-4, copied from K_4). +-20% kinetic convention (band over the S range 0.034-0.14 is for a dedicated sweep only). See nskinetics docs/reports/r14-r16-rate-laws-and-affinity-anchoring.md (2026-09-13).</t>
         </is>
       </c>
       <c r="K71" s="3" t="inlineStr">
@@ -3706,7 +3903,7 @@
         </is>
       </c>
       <c r="E72" s="3" t="n">
-        <v>1.416884904711885</v>
+        <v>0.7147832576024807</v>
       </c>
       <c r="F72" s="3" t="inlineStr">
         <is>
@@ -3714,15 +3911,19 @@
         </is>
       </c>
       <c r="G72" s="5" t="n">
-        <v>1.133507923769508</v>
+        <v>0.5718266060819847</v>
       </c>
       <c r="H72" s="5" t="n">
-        <v>1.416884904711885</v>
+        <v>0.7147832576024807</v>
       </c>
       <c r="I72" s="5" t="n">
-        <v>1.700261885654262</v>
-      </c>
-      <c r="J72" s="3" t="n"/>
+        <v>0.8577399091229768</v>
+      </c>
+      <c r="J72" s="3" t="inlineStr">
+        <is>
+          <t>opt_IRR: trial 1602 of kin_opt_ethanol_isobutanol_metabolic_split_12d_pi_log-tail_gp_rb0.001-4_ib0.75-1.5_aA_burden (anchor scenario A; build_opt_IRR_split12d_workbook.py)</t>
+        </is>
+      </c>
       <c r="K72" s="3" t="inlineStr">
         <is>
           <t>V406.nsk_kinetic_model._te.k_16 = x</t>
@@ -3769,7 +3970,7 @@
       </c>
       <c r="J73" s="3" t="inlineStr">
         <is>
-          <t>K_16 = 0.27 g/L: Aro10 (the rate-limiting decarboxylase of the lumped KDC + ADH step r16) KIV affinity, Km 8.5 mM (Kneen et al. 2011 FEBS J. 278:1842; BRENDA EC 4.1.1.43), anchored by ratio to r3's Pdc (Km 1.1 mM) exactly as K_13 was, with the molar-mass correction: (8.5/1.1) x 0.302 mM x 116.12 g/mol. r16 is irreversible Michaelis-Menten in KIV since 2026-09-13 (nskinetics b61360e; was 0.034, copied from K_6). +-20% kinetic convention (band 0.27-0.60 for Pdc Km 1.1-0.5 mM is for a dedicated sweep only). See nskinetics docs/reports/r14-r16-rate-laws-and-affinity-anchoring.md (2026-09-13). Since the 2026-09-15 nskinetics split of the lumped step, r16 is the Aro10 decarboxylation alone (KIV -&gt; isobutyraldehyde + CO2); the Adh6 aldehyde reduction is r17 (k_17, K_17, k_17r, K_17e, k_17ia, k_17ie).</t>
+          <t>opt_IRR: trial 1602 of kin_opt_ethanol_isobutanol_metabolic_split_12d_pi_log-tail_gp_rb0.001-4_ib0.75-1.5_aA_burden (anchor scenario A; build_opt_IRR_split12d_workbook.py) | template note: K_16 = 0.27 g/L: Aro10 (the rate-limiting decarboxylase of the lumped KDC + ADH step r16) KIV affinity, Km 8.5 mM (Kneen et al. 2011 FEBS J. 278:1842; BRENDA EC 4.1.1.43), anchored by ratio to r3's Pdc (Km 1.1 mM) exactly as K_13 was, with the molar-mass correction: (8.5/1.1) x 0.302 mM x 116.12 g/mol. r16 is irreversible Michaelis-Menten in KIV since 2026-09-13 (nskinetics b61360e; was 0.034, copied from K_6). +-20% kinetic convention (band 0.27-0.60 for Pdc Km 1.1-0.5 mM is for a dedicated sweep only). See nskinetics docs/reports/r14-r16-rate-laws-and-affinity-anchoring.md (2026-09-13). Since the 2026-09-15 nskinetics split of the lumped step, r16 is the Aro10 decarboxylation alone (KIV -&gt; isobutyraldehyde + CO2); the Adh6 aldehyde reduction is r17 (k_17, K_17, k_17r, K_17e, k_17ia, k_17ie).</t>
         </is>
       </c>
       <c r="K73" s="3" t="inlineStr">
@@ -3800,7 +4001,7 @@
         </is>
       </c>
       <c r="E74" t="n">
-        <v>0.1051981721819152</v>
+        <v>0.045</v>
       </c>
       <c r="F74" t="inlineStr">
         <is>
@@ -3808,17 +4009,17 @@
         </is>
       </c>
       <c r="G74" t="n">
-        <v>0.08415853774553214</v>
+        <v>0.036</v>
       </c>
       <c r="H74" t="n">
-        <v>0.1051981721819152</v>
+        <v>0.045</v>
       </c>
       <c r="I74" t="n">
-        <v>0.1262378066182982</v>
+        <v>0.054</v>
       </c>
       <c r="J74" t="inlineStr">
         <is>
-          <t>k_17ia (L/g): acetate cross-product exponential exp(-k_17ia*s_acetate) on the alcohol-forming step r17 -- the lumped r16's coefficient re-homed by the 2026-09-15 nskinetics split (value unchanged; symmetric with r6's k_6ia). The old k_16ia is declared inert (0) in the antimony.</t>
+          <t>opt_IRR: trial 1602 of kin_opt_ethanol_isobutanol_metabolic_split_12d_pi_log-tail_gp_rb0.001-4_ib0.75-1.5_aA_burden (anchor scenario A; build_opt_IRR_split12d_workbook.py) | template note: k_17ia (L/g): acetate cross-product exponential exp(-k_17ia*s_acetate) on the alcohol-forming step r17 -- the lumped r16's coefficient re-homed by the 2026-09-15 nskinetics split (value unchanged; symmetric with r6's k_6ia). The old k_16ia is declared inert (0) in the antimony.</t>
         </is>
       </c>
       <c r="K74" t="inlineStr">
@@ -3849,7 +4050,7 @@
         </is>
       </c>
       <c r="E75" t="n">
-        <v>0.004103299498839822</v>
+        <v>0.01618588154641622</v>
       </c>
       <c r="F75" t="inlineStr">
         <is>
@@ -3857,17 +4058,17 @@
         </is>
       </c>
       <c r="G75" t="n">
-        <v>0.003282639599071858</v>
+        <v>0.01294870523713298</v>
       </c>
       <c r="H75" t="n">
-        <v>0.004103299498839822</v>
+        <v>0.01618588154641622</v>
       </c>
       <c r="I75" t="n">
-        <v>0.004923959398607787</v>
+        <v>0.01942305785569947</v>
       </c>
       <c r="J75" t="inlineStr">
         <is>
-          <t>k_17ie (L/g): ethanol cross-product exponential exp(-k_17ie*s_EtOH) on the alcohol-forming step r17 -- the lumped r16's coefficient re-homed by the 2026-09-15 nskinetics split (value unchanged; symmetric with r6's k_6ie). The old k_16ie is declared inert (0) in the antimony.</t>
+          <t>opt_IRR: trial 1602 of kin_opt_ethanol_isobutanol_metabolic_split_12d_pi_log-tail_gp_rb0.001-4_ib0.75-1.5_aA_burden (anchor scenario A; build_opt_IRR_split12d_workbook.py) | template note: k_17ie (L/g): ethanol cross-product exponential exp(-k_17ie*s_EtOH) on the alcohol-forming step r17 -- the lumped r16's coefficient re-homed by the 2026-09-15 nskinetics split (value unchanged; symmetric with r6's k_6ie). The old k_16ie is declared inert (0) in the antimony.</t>
         </is>
       </c>
       <c r="K75" t="inlineStr">
@@ -3898,7 +4099,7 @@
         </is>
       </c>
       <c r="E76" t="n">
-        <v>44</v>
+        <v>2.154</v>
       </c>
       <c r="F76" t="inlineStr">
         <is>
@@ -3906,17 +4107,17 @@
         </is>
       </c>
       <c r="G76" t="n">
-        <v>35.2</v>
+        <v>1.7232</v>
       </c>
       <c r="H76" t="n">
-        <v>44</v>
+        <v>2.154</v>
       </c>
       <c r="I76" t="n">
-        <v>52.8</v>
+        <v>2.5848</v>
       </c>
       <c r="J76" t="inlineStr">
         <is>
-          <t>k_17 = 44 g/L/h: Adh6 (NADPH-dependent aldehyde reductase) capacity for the isobutyraldehyde -&gt; isobutanol step r17 of the 2026-09-15 nskinetics split of the lumped KDC + ADH step. A vmax grounded on the Adh6:Aro10 kcat ratio 296/19 (Adh6 296 s^-1 on 2-methylpropanal + NADPH, Larroy et al. 2002 Biochem. J. 361:163; Aro10 19 s^-1 on KIV, Kneen et al. 2011 FEBS J. 278:1842) x k_16's scenario-B value 2.82 g/L/h. CONSTITUTIVE (not a scenario toggle: the antimony default is 44 in every scenario, incl. A, where it is inert while k_16 = 0), set to keep Adh6 non-limiting at scenario-B flux. +-20 % kinetic convention.</t>
+          <t>opt_IRR: trial 1602 of kin_opt_ethanol_isobutanol_metabolic_split_12d_pi_log-tail_gp_rb0.001-4_ib0.75-1.5_aA_burden (anchor scenario A; build_opt_IRR_split12d_workbook.py) | template note: k_17 = 44 g/L/h: Adh6 (NADPH-dependent aldehyde reductase) capacity for the isobutyraldehyde -&gt; isobutanol step r17 of the 2026-09-15 nskinetics split of the lumped KDC + ADH step. A vmax grounded on the Adh6:Aro10 kcat ratio 296/19 (Adh6 296 s^-1 on 2-methylpropanal + NADPH, Larroy et al. 2002 Biochem. J. 361:163; Aro10 19 s^-1 on KIV, Kneen et al. 2011 FEBS J. 278:1842) x k_16's scenario-B value 2.82 g/L/h. CONSTITUTIVE (not a scenario toggle: the antimony default is 44 in every scenario, incl. A, where it is inert while k_16 = 0), set to keep Adh6 non-limiting at scenario-B flux. +-20 % kinetic convention.</t>
         </is>
       </c>
       <c r="K76" t="inlineStr">
@@ -3965,7 +4166,7 @@
       </c>
       <c r="J77" t="inlineStr">
         <is>
-          <t>K_17 = 0.0086 g/L: Adh6 isobutyraldehyde affinity, K_6 x (0.17/1.1) x (72.11/44.05) -- the Adh6:Adh1 aldehyde-affinity ratio (Adh6 branched-aldehyde Km 0.13-0.21 mM, midpoint 0.17 mM, Larroy et al. 2002 Biochem. J. 361:163; Adh1 acetaldehyde Km 1.1 mM, Ganzhorn et al. 1987 JBC 262:3754) applied to r6's fitted K_6 with the molar-mass correction (isobutyraldehyde 72.11 vs acetaldehyde 44.05 g/mol). nskinetics 2026-09-15 split. +-20 % kinetic convention.</t>
+          <t>opt_IRR: trial 1602 of kin_opt_ethanol_isobutanol_metabolic_split_12d_pi_log-tail_gp_rb0.001-4_ib0.75-1.5_aA_burden (anchor scenario A; build_opt_IRR_split12d_workbook.py) | template note: K_17 = 0.0086 g/L: Adh6 isobutyraldehyde affinity, K_6 x (0.17/1.1) x (72.11/44.05) -- the Adh6:Adh1 aldehyde-affinity ratio (Adh6 branched-aldehyde Km 0.13-0.21 mM, midpoint 0.17 mM, Larroy et al. 2002 Biochem. J. 361:163; Adh1 acetaldehyde Km 1.1 mM, Ganzhorn et al. 1987 JBC 262:3754) applied to r6's fitted K_6 with the molar-mass correction (isobutyraldehyde 72.11 vs acetaldehyde 44.05 g/mol). nskinetics 2026-09-15 split. +-20 % kinetic convention.</t>
         </is>
       </c>
       <c r="K77" t="inlineStr">
@@ -4014,7 +4215,7 @@
       </c>
       <c r="J78" t="inlineStr">
         <is>
-          <t>k_17r = 2.5e-4 (dimensionless): the r17 reverse-balance ratio, k_6r/50 -- r6's fitted Adh1 reverse balance scaled by Adh6's ~50-fold aldehyde-over-alcohol preference (Larroy et al. 2002 Biochem. J. 361:163). nskinetics 2026-09-15 split. +-20 % kinetic convention.</t>
+          <t>opt_IRR: trial 1602 of kin_opt_ethanol_isobutanol_metabolic_split_12d_pi_log-tail_gp_rb0.001-4_ib0.75-1.5_aA_burden (anchor scenario A; build_opt_IRR_split12d_workbook.py) | template note: k_17r = 2.5e-4 (dimensionless): the r17 reverse-balance ratio, k_6r/50 -- r6's fitted Adh1 reverse balance scaled by Adh6's ~50-fold aldehyde-over-alcohol preference (Larroy et al. 2002 Biochem. J. 361:163). nskinetics 2026-09-15 split. +-20 % kinetic convention.</t>
         </is>
       </c>
       <c r="K78" t="inlineStr">
@@ -4063,7 +4264,7 @@
       </c>
       <c r="J79" t="inlineStr">
         <is>
-          <t>K_17e = 0.020 (dimensionless): competitive isobutanol product term of r17, K_17 / Ki_IBO,model with Ki_IBO,model = 0.70 x 50 x 0.17 mM = 0.44 g/L isobutanol (the 0.70 is r6's own in-vitro -&gt; in-vivo transfer factor read off K_6/K_6e; 50 = Adh6's aldehyde-over-alcohol preference, Larroy et al. 2002). nskinetics 2026-09-15 split. +-20 % kinetic convention.</t>
+          <t>opt_IRR: trial 1602 of kin_opt_ethanol_isobutanol_metabolic_split_12d_pi_log-tail_gp_rb0.001-4_ib0.75-1.5_aA_burden (anchor scenario A; build_opt_IRR_split12d_workbook.py) | template note: K_17e = 0.020 (dimensionless): competitive isobutanol product term of r17, K_17 / Ki_IBO,model with Ki_IBO,model = 0.70 x 50 x 0.17 mM = 0.44 g/L isobutanol (the 0.70 is r6's own in-vitro -&gt; in-vivo transfer factor read off K_6/K_6e; 50 = Adh6's aldehyde-over-alcohol preference, Larroy et al. 2002). nskinetics 2026-09-15 split. +-20 % kinetic convention.</t>
         </is>
       </c>
       <c r="K79" t="inlineStr">

</xml_diff>